<commit_message>
Ny type split fra 1943
</commit_message>
<xml_diff>
--- a/Samlet_byggaktivitet_42-25.xlsx
+++ b/Samlet_byggaktivitet_42-25.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/emilnygaardeik/Documents/Industrial_Ecology/V_2026/MFA2/Project/TEP4290-project/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFC8D138-497A-1E47-AC2B-FE80905A04D5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{44295A62-B860-864C-9213-0450911BA7CB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="28800" windowHeight="18000" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="0" yWindow="500" windowWidth="28800" windowHeight="15940" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="BYGV05A" sheetId="2" r:id="rId1"/>
@@ -308,13 +308,13 @@
     <t>Tot</t>
   </si>
   <si>
-    <t>Ratio parcelhus</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ratio rekkehus </t>
-  </si>
-  <si>
-    <t>Ratio etage</t>
+    <t>Ratio_parcelhus</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ratio_rekkehus </t>
+  </si>
+  <si>
+    <t>Ratio_etage</t>
   </si>
 </sst>
 </file>

</xml_diff>